<commit_message>
:auto_rickshaw: CCA on restricted D1 (G1 larva + pupa + adult) on fungal com.
</commit_message>
<xml_diff>
--- a/data/derived_data/6_NMI_CCA/Dataset_1/CCA_NULL_ITS_D1_LarvaPupaAdult.xlsx
+++ b/data/derived_data/6_NMI_CCA/Dataset_1/CCA_NULL_ITS_D1_LarvaPupaAdult.xlsx
@@ -433,7 +433,7 @@
         <v>0.620062459347836</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6608</v>
+        <v>0.6674</v>
       </c>
     </row>
     <row r="4">
@@ -484,7 +484,7 @@
         <v>1.68879389821222</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1854</v>
+        <v>0.1838</v>
       </c>
     </row>
   </sheetData>

</xml_diff>